<commit_message>
the construction counts only what built the index the final runs read: Haiku's calls for the chunks in the graph with their share of the pass's time, the vectors, the Opus judgements the facet network learned from, the edge encoding and the steps with no model; the hardware row out; model names without publisher or snapshot date; CLAUDE.md: his words on it
</commit_message>
<xml_diff>
--- a/finished_data/construction.xlsx
+++ b/finished_data/construction.xlsx
@@ -11,8 +11,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="key" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'construction'!$A$1:$D$19</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'key'!$A$1:$B$19</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'construction'!$A$1:$D$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'key'!$A$1:$B$17</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -421,13 +421,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D19"/>
+  <dimension ref="A1:D17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="50" customWidth="1" min="1" max="1"/>
+    <col width="44" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
-    <col width="37" customWidth="1" min="3" max="3"/>
-    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="35" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -525,13 +525,13 @@
         <v>2982.903398909091</v>
       </c>
       <c r="D5" t="n">
-        <v>28682.1</v>
+        <v>12310.5062442175</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>nvidia/llama-nemotron-embed-1b-v2, texts embedded</t>
+          <t>llama-nemotron-embed-1b-v2, texts embedded</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -544,7 +544,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>nvidia/llama-nemotron-embed-1b-v2, tokens</t>
+          <t>llama-nemotron-embed-1b-v2, tokens</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -557,7 +557,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>nvidia/llama-nemotron-embed-1b-v2, seconds</t>
+          <t>llama-nemotron-embed-1b-v2, seconds</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -570,41 +570,41 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>claude-haiku-4-5-20251001, calls</t>
+          <t>claude-haiku-4-5, calls</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>11802</v>
+        <v>4878</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>claude-haiku-4-5-20251001, tokens in</t>
+          <t>claude-haiku-4-5, tokens in</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>22982655</v>
+        <v>8190926</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>claude-haiku-4-5-20251001, tokens out</t>
+          <t>claude-haiku-4-5, tokens out</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>10075140</v>
+        <v>1673729</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>claude-haiku-4-5-20251001, seconds</t>
+          <t>claude-haiku-4-5, seconds</t>
         </is>
       </c>
       <c r="D12" t="n">
-        <v>13644.6</v>
+        <v>3675.006244217499</v>
       </c>
     </row>
     <row r="13">
@@ -614,7 +614,7 @@
         </is>
       </c>
       <c r="D13" t="n">
-        <v>1720</v>
+        <v>920</v>
       </c>
     </row>
     <row r="14">
@@ -624,7 +624,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>58405680</v>
+        <v>31238028</v>
       </c>
     </row>
     <row r="15">
@@ -634,7 +634,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>65596</v>
+        <v>35071</v>
       </c>
     </row>
     <row r="16">
@@ -644,53 +644,21 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>2564.4</v>
+        <v>1458.6</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>4 candidate encoders, seconds</t>
+          <t>gte-reranker-modernbert-base, seconds</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>3227</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Alibaba-NLP/gte-reranker-modernbert-base, seconds</t>
-        </is>
-      </c>
-      <c r="D18" t="n">
         <v>3549.5</v>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>hardware</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>laptop CPU</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>desktop, NVIDIA GeForce GTX 1080 Ti</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>laptop; desktop, NVIDIA GeForce GTX 1080 Ti; Colab GPU; the model providers' services</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:D19"/>
+  <autoFilter ref="A1:D17"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -701,10 +669,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B19"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="50" customWidth="1" min="1" max="1"/>
+    <col width="44" customWidth="1" min="1" max="1"/>
     <col width="100" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
@@ -764,26 +732,26 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Time to build the index. Lucene builds it in memory at the start of each run. Vector's is the time to embed every record once. The artefact's is the time of each step of its build, added; the time between the steps is not counted.</t>
+          <t>Time to build the index that the final run read. Lucene builds it in memory at the start of each run. Vector's is the time to embed every record once. The artefact's is the time of each step of its build, added; the time between the steps is not counted.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>nvidia/llama-nemotron-embed-1b-v2, texts embedded</t>
+          <t>llama-nemotron-embed-1b-v2, texts embedded</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Texts that nvidia/llama-nemotron-embed-1b-v2 embedded in the build, one request each.</t>
+          <t>Texts that llama-nemotron-embed-1b-v2 embedded for the index, one request each.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>nvidia/llama-nemotron-embed-1b-v2, tokens</t>
+          <t>llama-nemotron-embed-1b-v2, tokens</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -795,60 +763,60 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>nvidia/llama-nemotron-embed-1b-v2, seconds</t>
+          <t>llama-nemotron-embed-1b-v2, seconds</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Time that nvidia/llama-nemotron-embed-1b-v2 worked in the build, from start to end.</t>
+          <t>Time that llama-nemotron-embed-1b-v2 worked for the index, from start to end.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>claude-haiku-4-5-20251001, calls</t>
+          <t>claude-haiku-4-5, calls</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Calls to claude-haiku-4-5-20251001 that the build's records count.</t>
+          <t>Calls to claude-haiku-4-5 for the index.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>claude-haiku-4-5-20251001, tokens in</t>
+          <t>claude-haiku-4-5, tokens in</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Tokens sent to claude-haiku-4-5-20251001 in the build.</t>
+          <t>Tokens sent to claude-haiku-4-5 for the index.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>claude-haiku-4-5-20251001, tokens out</t>
+          <t>claude-haiku-4-5, tokens out</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Tokens that claude-haiku-4-5-20251001 wrote in the build.</t>
+          <t>Tokens that claude-haiku-4-5 wrote for the index.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>claude-haiku-4-5-20251001, seconds</t>
+          <t>claude-haiku-4-5, seconds</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Time that claude-haiku-4-5-20251001 worked in the build, from start to end.</t>
+          <t>Time that claude-haiku-4-5 worked for the index: the time of the pass that wrote it, in the share of the calls' own time that the index's chunks took.</t>
         </is>
       </c>
     </row>
@@ -860,7 +828,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Calls to claude-opus-5 that the build's records count.</t>
+          <t>Calls to claude-opus-5 for the index.</t>
         </is>
       </c>
     </row>
@@ -872,7 +840,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Tokens sent to claude-opus-5 in the build.</t>
+          <t>Tokens sent to claude-opus-5 for the index.</t>
         </is>
       </c>
     </row>
@@ -884,7 +852,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Tokens that claude-opus-5 wrote in the build.</t>
+          <t>Tokens that claude-opus-5 wrote for the index.</t>
         </is>
       </c>
     </row>
@@ -896,48 +864,24 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Time that claude-opus-5 worked in the build, from start to end.</t>
+          <t>Time that claude-opus-5 worked for the index, from start to end.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>4 candidate encoders, seconds</t>
+          <t>gte-reranker-modernbert-base, seconds</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Time that 4 candidate encoders worked in the build, from start to end.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>Alibaba-NLP/gte-reranker-modernbert-base, seconds</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>Time that Alibaba-NLP/gte-reranker-modernbert-base worked in the build, from start to end.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>hardware</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>Where the index was built.</t>
+          <t>Time that gte-reranker-modernbert-base worked for the index, from start to end.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:B19"/>
+  <autoFilter ref="A1:B17"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
the construction's first column is called property
</commit_message>
<xml_diff>
--- a/finished_data/construction.xlsx
+++ b/finished_data/construction.xlsx
@@ -433,7 +433,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>thing</t>
+          <t>property</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -679,7 +679,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>thing</t>
+          <t>property</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">

</xml_diff>